<commit_message>
Correct B2 zero-candidate pause and clarify missing returns
</commit_message>
<xml_diff>
--- a/docs/stock_automl_runs/20261020_b2_recent_loss_resume_r55/B2_近5_10日亏损停手_R55_20261020.xlsx
+++ b/docs/stock_automl_runs/20261020_b2_recent_loss_resume_r55/B2_近5_10日亏损停手_R55_20261020.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R3410f3f21cd94a6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐月" sheetId="2" r:id="R5fb8ed2e79eb4b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐笔" sheetId="3" r:id="R8ee375bc166943b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Re35bd82c1d2e4343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐月" sheetId="2" r:id="Rcdd760e569c940a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐笔" sheetId="3" r:id="Rb06664bc6b454111"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -332,7 +332,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>原 B2 月模型；上月两窗口均亏则停。恢复方案仅在当月影子 D2 胜率超过 50% 后买下一笔。</x:v>
+        <x:v>原 B2 月模型；上月两窗口均亏或零候选则停。恢复方案仅在当月影子 D2 胜率超过 50% 后买下一笔。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26" customHeight="1">

</xml_diff>

<commit_message>
Replay B2 with prior 5 and 10 day return sum gate
</commit_message>
<xml_diff>
--- a/docs/stock_automl_runs/20261020_b2_recent_loss_resume_r55/B2_近5_10日亏损停手_R55_20261020.xlsx
+++ b/docs/stock_automl_runs/20261020_b2_recent_loss_resume_r55/B2_近5_10日亏损停手_R55_20261020.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Re35bd82c1d2e4343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐月" sheetId="2" r:id="Rcdd760e569c940a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐笔" sheetId="3" r:id="Rb06664bc6b454111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rce3872541b7d4524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐月" sheetId="2" r:id="R512bb4c956f64e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐笔" sheetId="3" r:id="R93dc44f0d4c2498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -499,6 +499,12 @@
       <x:c r="F11" s="7" t="str">
         <x:v>年化夏普</x:v>
       </x:c>
+      <x:c r="G11" s="7" t="str">
+        <x:v>D2费后胜率</x:v>
+      </x:c>
+      <x:c r="H11" s="7" t="str">
+        <x:v>D2费后笔均</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="21" customHeight="1">
       <x:c r="A12" s="3" t="str">
@@ -519,6 +525,12 @@
       <x:c r="F12" s="11" t="n">
         <x:v>-0.9055170423998936</x:v>
       </x:c>
+      <x:c r="G12" s="10" t="n">
+        <x:v>0.43462246777163904</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="n">
+        <x:v>-0.006627678425934701</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="21" customHeight="1">
       <x:c r="A13" s="3" t="str">
@@ -539,6 +551,12 @@
       <x:c r="F13" s="11" t="n">
         <x:v>0.34502401045532993</x:v>
       </x:c>
+      <x:c r="G13" s="10" t="n">
+        <x:v>0.465625</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="n">
+        <x:v>0.003938651800040063</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="21" customHeight="1">
       <x:c r="A14" s="3" t="str">
@@ -559,6 +577,12 @@
       <x:c r="F14" s="11" t="n">
         <x:v>-0.15764261618597117</x:v>
       </x:c>
+      <x:c r="G14" s="10" t="n">
+        <x:v>0.45232273838630804</x:v>
+      </x:c>
+      <x:c r="H14" s="9" t="n">
+        <x:v>-0.0008427991806323422</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="21" customHeight="1">
       <x:c r="A15" s="3" t="str">
@@ -579,6 +603,12 @@
       <x:c r="F15" s="11" t="n">
         <x:v>-0.6448454758818933</x:v>
       </x:c>
+      <x:c r="G15" s="10" t="n">
+        <x:v>0.44801980198019803</x:v>
+      </x:c>
+      <x:c r="H15" s="9" t="n">
+        <x:v>-0.004566818473456591</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="21" customHeight="1">
       <x:c r="A16" s="3" t="str">
@@ -599,6 +629,12 @@
       <x:c r="F16" s="11" t="n">
         <x:v>0.6224630364719124</x:v>
       </x:c>
+      <x:c r="G16" s="10" t="n">
+        <x:v>0.47863247863247865</x:v>
+      </x:c>
+      <x:c r="H16" s="9" t="n">
+        <x:v>0.006529963650340908</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="21" customHeight="1">
       <x:c r="A17" s="3" t="str">
@@ -619,6 +655,12 @@
       <x:c r="F17" s="11" t="n">
         <x:v>0.07066678866826075</x:v>
       </x:c>
+      <x:c r="G17" s="10" t="n">
+        <x:v>0.46405228758169936</x:v>
+      </x:c>
+      <x:c r="H17" s="9" t="n">
+        <x:v>0.001173254597543249</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="21" customHeight="1">
       <x:c r="A18" s="3" t="str">
@@ -639,6 +681,12 @@
       <x:c r="F18" s="11" t="n">
         <x:v>1.4800094333596874</x:v>
       </x:c>
+      <x:c r="G18" s="10" t="n">
+        <x:v>0.5155555555555555</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="n">
+        <x:v>0.011299556213424329</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="21" customHeight="1">
       <x:c r="A19" s="3" t="str">
@@ -659,6 +707,12 @@
       <x:c r="F19" s="11" t="n">
         <x:v>1.6423820078573186</x:v>
       </x:c>
+      <x:c r="G19" s="10" t="n">
+        <x:v>0.5161290322580645</x:v>
+      </x:c>
+      <x:c r="H19" s="9" t="n">
+        <x:v>0.013459255002799875</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="21" customHeight="1">
       <x:c r="A20" s="3" t="str">
@@ -679,6 +733,12 @@
       <x:c r="F20" s="11" t="n">
         <x:v>1.7049355073568746</x:v>
       </x:c>
+      <x:c r="G20" s="10" t="n">
+        <x:v>0.5175879396984925</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="n">
+        <x:v>0.013373021030953355</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="21" customHeight="1">
       <x:c r="A21" s="3" t="str">
@@ -699,6 +759,12 @@
       <x:c r="F21" s="11" t="n">
         <x:v>2.322813576045434</x:v>
       </x:c>
+      <x:c r="G21" s="10" t="n">
+        <x:v>0.525</x:v>
+      </x:c>
+      <x:c r="H21" s="9" t="n">
+        <x:v>0.01604799940002748</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="21" customHeight="1">
       <x:c r="A22" s="3" t="str">
@@ -719,6 +785,12 @@
       <x:c r="F22" s="11" t="n">
         <x:v>2.626871497119162</x:v>
       </x:c>
+      <x:c r="G22" s="10" t="n">
+        <x:v>0.5315315315315315</x:v>
+      </x:c>
+      <x:c r="H22" s="9" t="n">
+        <x:v>0.019035367534645322</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="21" customHeight="1">
       <x:c r="A23" s="3" t="str">
@@ -738,6 +810,12 @@
       </x:c>
       <x:c r="F23" s="11" t="n">
         <x:v>2.626871497119162</x:v>
+      </x:c>
+      <x:c r="G23" s="10" t="n">
+        <x:v>0.5315315315315315</x:v>
+      </x:c>
+      <x:c r="H23" s="9" t="n">
+        <x:v>0.019035367534645322</x:v>
       </x:c>
     </x:row>
     <x:row r="26">

</xml_diff>